<commit_message>
Update sold status for multiple POPs
</commit_message>
<xml_diff>
--- a/剩餘庫存清單.xlsx
+++ b/剩餘庫存清單.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="177">
   <si>
     <t>分類</t>
   </si>
@@ -542,6 +542,9 @@
   </si>
   <si>
     <t>The Mind Flayer (超大盒 奪心魔)</t>
+  </si>
+  <si>
+    <t>Sold</t>
   </si>
 </sst>
 </file>
@@ -1018,6 +1021,9 @@
       <c r="D10">
         <v>850</v>
       </c>
+      <c r="E10" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
@@ -1032,6 +1038,9 @@
       <c r="D11">
         <v>850</v>
       </c>
+      <c r="E11" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
@@ -1060,6 +1069,9 @@
       <c r="D13">
         <v>850</v>
       </c>
+      <c r="E13" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
@@ -1103,7 +1115,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -1117,7 +1129,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -1131,7 +1143,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -1145,7 +1157,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -1159,7 +1171,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:5">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -1173,7 +1185,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:5">
       <c r="A22" t="s">
         <v>6</v>
       </c>
@@ -1187,7 +1199,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
         <v>6</v>
       </c>
@@ -1201,7 +1213,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:5">
       <c r="A24" t="s">
         <v>6</v>
       </c>
@@ -1214,8 +1226,11 @@
       <c r="D24">
         <v>750</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="E24" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
       <c r="A25" t="s">
         <v>6</v>
       </c>
@@ -1229,7 +1244,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:5">
       <c r="A26" t="s">
         <v>7</v>
       </c>
@@ -1243,7 +1258,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:5">
       <c r="A27" t="s">
         <v>6</v>
       </c>
@@ -1257,7 +1272,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:5">
       <c r="A28" t="s">
         <v>6</v>
       </c>
@@ -1271,7 +1286,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:5">
       <c r="A29" t="s">
         <v>6</v>
       </c>
@@ -1285,7 +1300,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:5">
       <c r="A30" t="s">
         <v>6</v>
       </c>
@@ -1299,7 +1314,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:5">
       <c r="A31" t="s">
         <v>6</v>
       </c>
@@ -1313,7 +1328,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:5">
       <c r="A32" t="s">
         <v>6</v>
       </c>
@@ -1327,7 +1342,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:5">
       <c r="A33" t="s">
         <v>6</v>
       </c>
@@ -1341,7 +1356,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:5">
       <c r="A34" t="s">
         <v>6</v>
       </c>
@@ -1355,7 +1370,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:5">
       <c r="A35" t="s">
         <v>6</v>
       </c>
@@ -1369,7 +1384,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:5">
       <c r="A36" t="s">
         <v>6</v>
       </c>
@@ -1383,7 +1398,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:5">
       <c r="A37" t="s">
         <v>6</v>
       </c>
@@ -1397,7 +1412,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:5">
       <c r="A38" t="s">
         <v>6</v>
       </c>
@@ -1411,7 +1426,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:5">
       <c r="A39" t="s">
         <v>6</v>
       </c>
@@ -1424,8 +1439,11 @@
       <c r="D39">
         <v>500</v>
       </c>
-    </row>
-    <row r="40" spans="1:4">
+      <c r="E39" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
       <c r="A40" t="s">
         <v>6</v>
       </c>
@@ -1439,7 +1457,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:5">
       <c r="A41" t="s">
         <v>6</v>
       </c>
@@ -1453,7 +1471,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:5">
       <c r="A42" t="s">
         <v>6</v>
       </c>
@@ -1467,7 +1485,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:5">
       <c r="A43" t="s">
         <v>6</v>
       </c>
@@ -1480,8 +1498,11 @@
       <c r="D43">
         <v>500</v>
       </c>
-    </row>
-    <row r="44" spans="1:4">
+      <c r="E43" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
       <c r="A44" t="s">
         <v>6</v>
       </c>
@@ -1495,7 +1516,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:5">
       <c r="A45" t="s">
         <v>6</v>
       </c>
@@ -1509,7 +1530,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:5">
       <c r="A46" t="s">
         <v>6</v>
       </c>
@@ -1522,8 +1543,11 @@
       <c r="D46">
         <v>500</v>
       </c>
-    </row>
-    <row r="47" spans="1:4">
+      <c r="E46" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
       <c r="A47" t="s">
         <v>6</v>
       </c>
@@ -1537,7 +1561,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
+    <row r="48" spans="1:5">
       <c r="A48" t="s">
         <v>6</v>
       </c>
@@ -1551,7 +1575,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
+    <row r="49" spans="1:5">
       <c r="A49" t="s">
         <v>6</v>
       </c>
@@ -1565,7 +1589,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:5">
       <c r="A50" t="s">
         <v>6</v>
       </c>
@@ -1579,7 +1603,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:5">
       <c r="A51" t="s">
         <v>7</v>
       </c>
@@ -1593,7 +1617,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:5">
       <c r="A52" t="s">
         <v>6</v>
       </c>
@@ -1607,7 +1631,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:5">
       <c r="A53" t="s">
         <v>6</v>
       </c>
@@ -1621,7 +1645,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:5">
       <c r="A54" t="s">
         <v>6</v>
       </c>
@@ -1635,7 +1659,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:5">
       <c r="A55" t="s">
         <v>6</v>
       </c>
@@ -1649,7 +1673,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:5">
       <c r="A56" t="s">
         <v>6</v>
       </c>
@@ -1663,7 +1687,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="57" spans="1:4">
+    <row r="57" spans="1:5">
       <c r="A57" t="s">
         <v>6</v>
       </c>
@@ -1677,7 +1701,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="58" spans="1:4">
+    <row r="58" spans="1:5">
       <c r="A58" t="s">
         <v>6</v>
       </c>
@@ -1691,7 +1715,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
+    <row r="59" spans="1:5">
       <c r="A59" t="s">
         <v>6</v>
       </c>
@@ -1704,8 +1728,11 @@
       <c r="D59">
         <v>500</v>
       </c>
-    </row>
-    <row r="60" spans="1:4">
+      <c r="E59" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
       <c r="A60" t="s">
         <v>6</v>
       </c>
@@ -1719,7 +1746,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="61" spans="1:4">
+    <row r="61" spans="1:5">
       <c r="A61" t="s">
         <v>6</v>
       </c>
@@ -1733,7 +1760,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="62" spans="1:4">
+    <row r="62" spans="1:5">
       <c r="A62" t="s">
         <v>6</v>
       </c>
@@ -1747,7 +1774,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="63" spans="1:4">
+    <row r="63" spans="1:5">
       <c r="A63" t="s">
         <v>6</v>
       </c>
@@ -1761,7 +1788,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="64" spans="1:4">
+    <row r="64" spans="1:5">
       <c r="A64" t="s">
         <v>6</v>
       </c>
@@ -1775,7 +1802,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="65" spans="1:4">
+    <row r="65" spans="1:5">
       <c r="A65" t="s">
         <v>6</v>
       </c>
@@ -1789,7 +1816,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="66" spans="1:4">
+    <row r="66" spans="1:5">
       <c r="A66" t="s">
         <v>6</v>
       </c>
@@ -1803,7 +1830,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="67" spans="1:4">
+    <row r="67" spans="1:5">
       <c r="A67" t="s">
         <v>6</v>
       </c>
@@ -1817,7 +1844,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="68" spans="1:4">
+    <row r="68" spans="1:5">
       <c r="A68" t="s">
         <v>6</v>
       </c>
@@ -1831,7 +1858,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="69" spans="1:4">
+    <row r="69" spans="1:5">
       <c r="A69" t="s">
         <v>6</v>
       </c>
@@ -1844,8 +1871,11 @@
       <c r="D69">
         <v>500</v>
       </c>
-    </row>
-    <row r="70" spans="1:4">
+      <c r="E69" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
       <c r="A70" t="s">
         <v>6</v>
       </c>
@@ -1859,7 +1889,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="71" spans="1:4">
+    <row r="71" spans="1:5">
       <c r="A71" t="s">
         <v>6</v>
       </c>
@@ -1873,7 +1903,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="72" spans="1:4">
+    <row r="72" spans="1:5">
       <c r="A72" t="s">
         <v>6</v>
       </c>
@@ -1887,7 +1917,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="73" spans="1:4">
+    <row r="73" spans="1:5">
       <c r="A73" t="s">
         <v>6</v>
       </c>
@@ -1901,7 +1931,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="74" spans="1:4">
+    <row r="74" spans="1:5">
       <c r="A74" t="s">
         <v>6</v>
       </c>
@@ -1915,7 +1945,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="75" spans="1:4">
+    <row r="75" spans="1:5">
       <c r="A75" t="s">
         <v>6</v>
       </c>
@@ -1929,7 +1959,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="76" spans="1:4">
+    <row r="76" spans="1:5">
       <c r="A76" t="s">
         <v>6</v>
       </c>
@@ -1943,7 +1973,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="77" spans="1:4">
+    <row r="77" spans="1:5">
       <c r="A77" t="s">
         <v>6</v>
       </c>
@@ -1957,7 +1987,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="78" spans="1:4">
+    <row r="78" spans="1:5">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -1971,7 +2001,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="79" spans="1:4">
+    <row r="79" spans="1:5">
       <c r="A79" t="s">
         <v>8</v>
       </c>
@@ -1985,7 +2015,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="80" spans="1:4">
+    <row r="80" spans="1:5">
       <c r="A80" t="s">
         <v>8</v>
       </c>
@@ -1999,7 +2029,7 @@
         <v>1750</v>
       </c>
     </row>
-    <row r="81" spans="1:4">
+    <row r="81" spans="1:5">
       <c r="A81" t="s">
         <v>8</v>
       </c>
@@ -2013,7 +2043,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="82" spans="1:4">
+    <row r="82" spans="1:5">
       <c r="A82" t="s">
         <v>8</v>
       </c>
@@ -2027,7 +2057,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="83" spans="1:4">
+    <row r="83" spans="1:5">
       <c r="A83" t="s">
         <v>8</v>
       </c>
@@ -2041,7 +2071,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="84" spans="1:4">
+    <row r="84" spans="1:5">
       <c r="A84" t="s">
         <v>8</v>
       </c>
@@ -2055,7 +2085,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="85" spans="1:4">
+    <row r="85" spans="1:5">
       <c r="A85" t="s">
         <v>8</v>
       </c>
@@ -2069,7 +2099,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="86" spans="1:4">
+    <row r="86" spans="1:5">
       <c r="A86" t="s">
         <v>8</v>
       </c>
@@ -2083,7 +2113,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="87" spans="1:4">
+    <row r="87" spans="1:5">
       <c r="A87" t="s">
         <v>8</v>
       </c>
@@ -2097,7 +2127,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="88" spans="1:4">
+    <row r="88" spans="1:5">
       <c r="A88" t="s">
         <v>8</v>
       </c>
@@ -2109,6 +2139,9 @@
       </c>
       <c r="D88">
         <v>500</v>
+      </c>
+      <c r="E88" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark POP 1303 as sold
</commit_message>
<xml_diff>
--- a/剩餘庫存清單.xlsx
+++ b/剩餘庫存清單.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="177">
   <si>
     <t>分類</t>
   </si>
@@ -1529,6 +1529,9 @@
       <c r="D45">
         <v>500</v>
       </c>
+      <c r="E45" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">

</xml_diff>